<commit_message>
se conectan bodega con entrada material
</commit_message>
<xml_diff>
--- a/materiales.xlsx
+++ b/materiales.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Bodeg\Cointeca\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D727FB7F-CD2C-4792-AEA6-58A43AD8D4A2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0C8FC609-FD05-4503-A864-CC778332DDA5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{E2040FC4-B0BA-4472-B1A9-67F29144F1F8}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="555" uniqueCount="362">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="713" uniqueCount="361">
   <si>
     <t>ITEM</t>
   </si>
@@ -485,9 +485,6 @@
     <t>Grapa Pistola</t>
   </si>
   <si>
-    <t>Desmonte Collarines</t>
-  </si>
-  <si>
     <t>Cable Aluminio Acsr 4/0 (Desmonte)</t>
   </si>
   <si>
@@ -1115,16 +1112,16 @@
     <t>CONTRAMARCO</t>
   </si>
   <si>
-    <t>UNIDAD</t>
-  </si>
-  <si>
     <t>UN</t>
   </si>
   <si>
-    <t>M</t>
-  </si>
-  <si>
-    <t>Un</t>
+    <t>KG</t>
+  </si>
+  <si>
+    <t>MT</t>
+  </si>
+  <si>
+    <t>CANTIDAD</t>
   </si>
 </sst>
 </file>
@@ -1502,10 +1499,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F33D0EAE-A27C-40D9-8B5C-2DBEAC1A1F5E}">
-  <dimension ref="A1:E357"/>
+  <dimension ref="A1:E356"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="44.28515625" customWidth="1"/>
+    <col min="2" max="2" width="58.140625" customWidth="1"/>
     <col min="3" max="3" width="11" customWidth="1"/>
   </cols>
   <sheetData>
@@ -1517,7 +1514,7 @@
         <v>1</v>
       </c>
       <c r="C1" t="s">
-        <v>358</v>
+        <v>360</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
@@ -1527,6 +1524,9 @@
       <c r="B2" s="1" t="s">
         <v>2</v>
       </c>
+      <c r="C2" t="s">
+        <v>357</v>
+      </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3">
@@ -1535,6 +1535,9 @@
       <c r="B3" s="1" t="s">
         <v>3</v>
       </c>
+      <c r="C3" t="s">
+        <v>357</v>
+      </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4">
@@ -1543,6 +1546,9 @@
       <c r="B4" s="1" t="s">
         <v>4</v>
       </c>
+      <c r="C4" t="s">
+        <v>357</v>
+      </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5">
@@ -1551,6 +1557,9 @@
       <c r="B5" s="1" t="s">
         <v>5</v>
       </c>
+      <c r="C5" t="s">
+        <v>357</v>
+      </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6">
@@ -1559,6 +1568,9 @@
       <c r="B6" s="1" t="s">
         <v>6</v>
       </c>
+      <c r="C6" t="s">
+        <v>357</v>
+      </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7">
@@ -1567,6 +1579,9 @@
       <c r="B7" s="1" t="s">
         <v>7</v>
       </c>
+      <c r="C7" t="s">
+        <v>357</v>
+      </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8">
@@ -1575,6 +1590,9 @@
       <c r="B8" s="1" t="s">
         <v>8</v>
       </c>
+      <c r="C8" t="s">
+        <v>357</v>
+      </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9">
@@ -1583,6 +1601,9 @@
       <c r="B9" s="1" t="s">
         <v>9</v>
       </c>
+      <c r="C9" t="s">
+        <v>357</v>
+      </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A10">
@@ -1591,6 +1612,9 @@
       <c r="B10" s="1" t="s">
         <v>10</v>
       </c>
+      <c r="C10" t="s">
+        <v>357</v>
+      </c>
       <c r="E10" s="2"/>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.25">
@@ -1600,6 +1624,9 @@
       <c r="B11" s="1" t="s">
         <v>11</v>
       </c>
+      <c r="C11" t="s">
+        <v>357</v>
+      </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A12">
@@ -1608,6 +1635,9 @@
       <c r="B12" s="1" t="s">
         <v>12</v>
       </c>
+      <c r="C12" t="s">
+        <v>357</v>
+      </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A13">
@@ -1616,6 +1646,9 @@
       <c r="B13" s="1" t="s">
         <v>13</v>
       </c>
+      <c r="C13" t="s">
+        <v>357</v>
+      </c>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A14">
@@ -1624,6 +1657,9 @@
       <c r="B14" s="1" t="s">
         <v>14</v>
       </c>
+      <c r="C14" t="s">
+        <v>357</v>
+      </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A15">
@@ -1632,6 +1668,9 @@
       <c r="B15" s="1" t="s">
         <v>15</v>
       </c>
+      <c r="C15" t="s">
+        <v>357</v>
+      </c>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A16">
@@ -1640,1346 +1679,1784 @@
       <c r="B16" s="1" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C16" t="s">
+        <v>357</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A17">
         <v>16</v>
       </c>
       <c r="B17" s="1" t="s">
         <v>17</v>
       </c>
-    </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C17" t="s">
+        <v>357</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A18">
         <v>17</v>
       </c>
       <c r="B18" s="1" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C18" t="s">
+        <v>357</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A19">
         <v>18</v>
       </c>
       <c r="B19" s="1" t="s">
         <v>19</v>
       </c>
-    </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C19" t="s">
+        <v>357</v>
+      </c>
+    </row>
+    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A20">
         <v>19</v>
       </c>
       <c r="B20" s="1" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C20" t="s">
+        <v>357</v>
+      </c>
+    </row>
+    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A21">
         <v>20</v>
       </c>
       <c r="B21" s="1" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="22" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C21" t="s">
+        <v>357</v>
+      </c>
+    </row>
+    <row r="22" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A22">
         <v>21</v>
       </c>
       <c r="B22" s="1" t="s">
         <v>22</v>
       </c>
-    </row>
-    <row r="23" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C22" t="s">
+        <v>357</v>
+      </c>
+    </row>
+    <row r="23" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A23">
         <v>22</v>
       </c>
       <c r="B23" s="1" t="s">
         <v>23</v>
       </c>
-    </row>
-    <row r="24" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C23" t="s">
+        <v>357</v>
+      </c>
+    </row>
+    <row r="24" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A24">
         <v>23</v>
       </c>
       <c r="B24" s="1" t="s">
         <v>24</v>
       </c>
-    </row>
-    <row r="25" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C24" t="s">
+        <v>357</v>
+      </c>
+    </row>
+    <row r="25" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A25">
         <v>24</v>
       </c>
       <c r="B25" s="1" t="s">
         <v>25</v>
       </c>
-    </row>
-    <row r="26" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C25" t="s">
+        <v>357</v>
+      </c>
+    </row>
+    <row r="26" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A26">
         <v>25</v>
       </c>
       <c r="B26" s="1" t="s">
         <v>26</v>
       </c>
-    </row>
-    <row r="27" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C26" t="s">
+        <v>359</v>
+      </c>
+    </row>
+    <row r="27" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A27">
         <v>26</v>
       </c>
       <c r="B27" s="1" t="s">
         <v>27</v>
       </c>
-    </row>
-    <row r="28" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C27" t="s">
+        <v>359</v>
+      </c>
+    </row>
+    <row r="28" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A28">
         <v>27</v>
       </c>
       <c r="B28" s="1" t="s">
         <v>28</v>
       </c>
-    </row>
-    <row r="29" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C28" t="s">
+        <v>359</v>
+      </c>
+    </row>
+    <row r="29" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A29">
         <v>28</v>
       </c>
       <c r="B29" s="1" t="s">
         <v>29</v>
       </c>
-    </row>
-    <row r="30" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C29" t="s">
+        <v>358</v>
+      </c>
+    </row>
+    <row r="30" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A30">
         <v>29</v>
       </c>
       <c r="B30" s="1" t="s">
         <v>30</v>
       </c>
-    </row>
-    <row r="31" spans="1:2" ht="30" x14ac:dyDescent="0.25">
+      <c r="C30" t="s">
+        <v>357</v>
+      </c>
+    </row>
+    <row r="31" spans="1:3" ht="30" x14ac:dyDescent="0.25">
       <c r="A31">
         <v>30</v>
       </c>
       <c r="B31" s="1" t="s">
         <v>31</v>
       </c>
-    </row>
-    <row r="32" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C31" t="s">
+        <v>357</v>
+      </c>
+    </row>
+    <row r="32" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A32">
         <v>31</v>
       </c>
       <c r="B32" s="1" t="s">
         <v>32</v>
       </c>
-    </row>
-    <row r="33" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C32" t="s">
+        <v>357</v>
+      </c>
+    </row>
+    <row r="33" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A33">
         <v>32</v>
       </c>
       <c r="B33" s="1" t="s">
         <v>33</v>
       </c>
-    </row>
-    <row r="34" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C33" t="s">
+        <v>357</v>
+      </c>
+    </row>
+    <row r="34" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A34">
         <v>33</v>
       </c>
       <c r="B34" s="1" t="s">
         <v>34</v>
       </c>
-    </row>
-    <row r="35" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C34" t="s">
+        <v>357</v>
+      </c>
+    </row>
+    <row r="35" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A35">
         <v>34</v>
       </c>
       <c r="B35" s="1" t="s">
         <v>35</v>
       </c>
-    </row>
-    <row r="36" spans="1:2" ht="30" x14ac:dyDescent="0.25">
+      <c r="C35" t="s">
+        <v>357</v>
+      </c>
+    </row>
+    <row r="36" spans="1:3" ht="30" x14ac:dyDescent="0.25">
       <c r="A36">
         <v>35</v>
       </c>
       <c r="B36" s="1" t="s">
         <v>36</v>
       </c>
-    </row>
-    <row r="37" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C36" t="s">
+        <v>357</v>
+      </c>
+    </row>
+    <row r="37" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A37">
         <v>36</v>
       </c>
       <c r="B37" s="1" t="s">
         <v>37</v>
       </c>
-    </row>
-    <row r="38" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C37" t="s">
+        <v>357</v>
+      </c>
+    </row>
+    <row r="38" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A38">
         <v>37</v>
       </c>
       <c r="B38" s="1" t="s">
         <v>38</v>
       </c>
-    </row>
-    <row r="39" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C38" t="s">
+        <v>359</v>
+      </c>
+    </row>
+    <row r="39" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A39">
         <v>38</v>
       </c>
       <c r="B39" s="1" t="s">
         <v>39</v>
       </c>
-    </row>
-    <row r="40" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C39" t="s">
+        <v>359</v>
+      </c>
+    </row>
+    <row r="40" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A40">
         <v>39</v>
       </c>
       <c r="B40" s="1" t="s">
         <v>40</v>
       </c>
-    </row>
-    <row r="41" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C40" t="s">
+        <v>359</v>
+      </c>
+    </row>
+    <row r="41" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A41">
         <v>40</v>
       </c>
       <c r="B41" s="1" t="s">
         <v>41</v>
       </c>
-    </row>
-    <row r="42" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C41" t="s">
+        <v>359</v>
+      </c>
+    </row>
+    <row r="42" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A42">
         <v>41</v>
       </c>
       <c r="B42" s="1" t="s">
         <v>42</v>
       </c>
-    </row>
-    <row r="43" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C42" t="s">
+        <v>359</v>
+      </c>
+    </row>
+    <row r="43" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A43">
         <v>42</v>
       </c>
       <c r="B43" s="1" t="s">
         <v>43</v>
       </c>
-    </row>
-    <row r="44" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C43" t="s">
+        <v>359</v>
+      </c>
+    </row>
+    <row r="44" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A44">
         <v>43</v>
       </c>
       <c r="B44" s="1" t="s">
         <v>44</v>
       </c>
-    </row>
-    <row r="45" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C44" t="s">
+        <v>359</v>
+      </c>
+    </row>
+    <row r="45" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A45">
         <v>44</v>
       </c>
       <c r="B45" s="1" t="s">
         <v>45</v>
       </c>
-    </row>
-    <row r="46" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C45" t="s">
+        <v>357</v>
+      </c>
+    </row>
+    <row r="46" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A46">
         <v>45</v>
       </c>
       <c r="B46" s="1" t="s">
         <v>46</v>
       </c>
-    </row>
-    <row r="47" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C46" t="s">
+        <v>359</v>
+      </c>
+    </row>
+    <row r="47" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A47">
         <v>46</v>
       </c>
       <c r="B47" s="1" t="s">
         <v>47</v>
       </c>
-    </row>
-    <row r="48" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C47" t="s">
+        <v>357</v>
+      </c>
+    </row>
+    <row r="48" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A48">
         <v>47</v>
       </c>
       <c r="B48" s="1" t="s">
         <v>48</v>
       </c>
-    </row>
-    <row r="49" spans="1:2" ht="30" x14ac:dyDescent="0.25">
+      <c r="C48" t="s">
+        <v>357</v>
+      </c>
+    </row>
+    <row r="49" spans="1:3" ht="30" x14ac:dyDescent="0.25">
       <c r="A49">
         <v>48</v>
       </c>
       <c r="B49" s="1" t="s">
         <v>49</v>
       </c>
-    </row>
-    <row r="50" spans="1:2" ht="30" x14ac:dyDescent="0.25">
+      <c r="C49" t="s">
+        <v>359</v>
+      </c>
+    </row>
+    <row r="50" spans="1:3" ht="30" x14ac:dyDescent="0.25">
       <c r="A50">
         <v>49</v>
       </c>
       <c r="B50" s="1" t="s">
         <v>50</v>
       </c>
-    </row>
-    <row r="51" spans="1:2" ht="30" x14ac:dyDescent="0.25">
+      <c r="C50" t="s">
+        <v>359</v>
+      </c>
+    </row>
+    <row r="51" spans="1:3" ht="30" x14ac:dyDescent="0.25">
       <c r="A51">
         <v>50</v>
       </c>
       <c r="B51" s="1" t="s">
         <v>51</v>
       </c>
-    </row>
-    <row r="52" spans="1:2" ht="30" x14ac:dyDescent="0.25">
+      <c r="C51" t="s">
+        <v>359</v>
+      </c>
+    </row>
+    <row r="52" spans="1:3" ht="30" x14ac:dyDescent="0.25">
       <c r="A52">
         <v>51</v>
       </c>
       <c r="B52" s="1" t="s">
         <v>52</v>
       </c>
-    </row>
-    <row r="53" spans="1:2" ht="30" x14ac:dyDescent="0.25">
+      <c r="C52" t="s">
+        <v>359</v>
+      </c>
+    </row>
+    <row r="53" spans="1:3" ht="30" x14ac:dyDescent="0.25">
       <c r="A53">
         <v>52</v>
       </c>
       <c r="B53" s="1" t="s">
         <v>53</v>
       </c>
-    </row>
-    <row r="54" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C53" t="s">
+        <v>359</v>
+      </c>
+    </row>
+    <row r="54" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A54">
         <v>53</v>
       </c>
       <c r="B54" s="1" t="s">
         <v>54</v>
       </c>
-    </row>
-    <row r="55" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C54" t="s">
+        <v>359</v>
+      </c>
+    </row>
+    <row r="55" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A55">
         <v>54</v>
       </c>
       <c r="B55" s="1" t="s">
         <v>55</v>
       </c>
-    </row>
-    <row r="56" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C55" t="s">
+        <v>357</v>
+      </c>
+    </row>
+    <row r="56" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A56">
         <v>55</v>
       </c>
       <c r="B56" s="1" t="s">
         <v>56</v>
       </c>
-    </row>
-    <row r="57" spans="1:2" ht="30" x14ac:dyDescent="0.25">
+      <c r="C56" t="s">
+        <v>357</v>
+      </c>
+    </row>
+    <row r="57" spans="1:3" ht="30" x14ac:dyDescent="0.25">
       <c r="A57">
         <v>56</v>
       </c>
       <c r="B57" s="1" t="s">
         <v>57</v>
       </c>
-    </row>
-    <row r="58" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C57" t="s">
+        <v>357</v>
+      </c>
+    </row>
+    <row r="58" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A58">
         <v>57</v>
       </c>
       <c r="B58" s="1" t="s">
         <v>58</v>
       </c>
-    </row>
-    <row r="59" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C58" t="s">
+        <v>357</v>
+      </c>
+    </row>
+    <row r="59" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A59">
         <v>58</v>
       </c>
       <c r="B59" s="1" t="s">
         <v>59</v>
       </c>
-    </row>
-    <row r="60" spans="1:2" ht="30" x14ac:dyDescent="0.25">
+      <c r="C59" t="s">
+        <v>357</v>
+      </c>
+    </row>
+    <row r="60" spans="1:3" ht="30" x14ac:dyDescent="0.25">
       <c r="A60">
         <v>59</v>
       </c>
       <c r="B60" s="1" t="s">
         <v>60</v>
       </c>
-    </row>
-    <row r="61" spans="1:2" ht="30" x14ac:dyDescent="0.25">
+      <c r="C60" t="s">
+        <v>357</v>
+      </c>
+    </row>
+    <row r="61" spans="1:3" ht="30" x14ac:dyDescent="0.25">
       <c r="A61">
         <v>60</v>
       </c>
       <c r="B61" s="1" t="s">
         <v>61</v>
       </c>
-    </row>
-    <row r="62" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C61" t="s">
+        <v>357</v>
+      </c>
+    </row>
+    <row r="62" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A62">
         <v>61</v>
       </c>
       <c r="B62" s="1" t="s">
         <v>62</v>
       </c>
-    </row>
-    <row r="63" spans="1:2" ht="30" x14ac:dyDescent="0.25">
+      <c r="C62" t="s">
+        <v>357</v>
+      </c>
+    </row>
+    <row r="63" spans="1:3" ht="30" x14ac:dyDescent="0.25">
       <c r="A63">
         <v>62</v>
       </c>
       <c r="B63" s="1" t="s">
         <v>63</v>
       </c>
-    </row>
-    <row r="64" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C63" t="s">
+        <v>357</v>
+      </c>
+    </row>
+    <row r="64" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A64">
         <v>63</v>
       </c>
       <c r="B64" s="1" t="s">
         <v>64</v>
       </c>
-    </row>
-    <row r="65" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C64" t="s">
+        <v>357</v>
+      </c>
+    </row>
+    <row r="65" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A65">
         <v>64</v>
       </c>
       <c r="B65" s="1" t="s">
         <v>65</v>
       </c>
-    </row>
-    <row r="66" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C65" t="s">
+        <v>357</v>
+      </c>
+    </row>
+    <row r="66" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A66">
         <v>65</v>
       </c>
       <c r="B66" s="1" t="s">
         <v>66</v>
       </c>
-    </row>
-    <row r="67" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C66" t="s">
+        <v>357</v>
+      </c>
+    </row>
+    <row r="67" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A67">
         <v>66</v>
       </c>
       <c r="B67" s="1" t="s">
         <v>67</v>
       </c>
-    </row>
-    <row r="68" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C67" t="s">
+        <v>357</v>
+      </c>
+    </row>
+    <row r="68" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A68">
         <v>67</v>
       </c>
       <c r="B68" s="1" t="s">
         <v>68</v>
       </c>
-    </row>
-    <row r="69" spans="1:2" ht="45" x14ac:dyDescent="0.25">
+      <c r="C68" t="s">
+        <v>357</v>
+      </c>
+    </row>
+    <row r="69" spans="1:3" ht="45" x14ac:dyDescent="0.25">
       <c r="A69">
         <v>68</v>
       </c>
       <c r="B69" s="1" t="s">
         <v>69</v>
       </c>
-    </row>
-    <row r="70" spans="1:2" ht="45" x14ac:dyDescent="0.25">
+      <c r="C69" t="s">
+        <v>357</v>
+      </c>
+    </row>
+    <row r="70" spans="1:3" ht="45" x14ac:dyDescent="0.25">
       <c r="A70">
         <v>69</v>
       </c>
       <c r="B70" s="1" t="s">
         <v>70</v>
       </c>
-    </row>
-    <row r="71" spans="1:2" ht="30" x14ac:dyDescent="0.25">
+      <c r="C70" t="s">
+        <v>357</v>
+      </c>
+    </row>
+    <row r="71" spans="1:3" ht="30" x14ac:dyDescent="0.25">
       <c r="A71">
         <v>70</v>
       </c>
       <c r="B71" s="1" t="s">
         <v>71</v>
       </c>
-    </row>
-    <row r="72" spans="1:2" ht="30" x14ac:dyDescent="0.25">
+      <c r="C71" t="s">
+        <v>357</v>
+      </c>
+    </row>
+    <row r="72" spans="1:3" ht="30" x14ac:dyDescent="0.25">
       <c r="A72">
         <v>71</v>
       </c>
       <c r="B72" s="1" t="s">
         <v>72</v>
       </c>
-    </row>
-    <row r="73" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C72" t="s">
+        <v>357</v>
+      </c>
+    </row>
+    <row r="73" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A73">
         <v>72</v>
       </c>
       <c r="B73" s="1" t="s">
         <v>73</v>
       </c>
-    </row>
-    <row r="74" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C73" t="s">
+        <v>357</v>
+      </c>
+    </row>
+    <row r="74" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A74">
         <v>73</v>
       </c>
       <c r="B74" s="1" t="s">
         <v>74</v>
       </c>
-    </row>
-    <row r="75" spans="1:2" ht="30" x14ac:dyDescent="0.25">
+      <c r="C74" t="s">
+        <v>357</v>
+      </c>
+    </row>
+    <row r="75" spans="1:3" ht="30" x14ac:dyDescent="0.25">
       <c r="A75">
         <v>74</v>
       </c>
       <c r="B75" s="1" t="s">
         <v>75</v>
       </c>
-    </row>
-    <row r="76" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C75" t="s">
+        <v>357</v>
+      </c>
+    </row>
+    <row r="76" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A76">
         <v>75</v>
       </c>
       <c r="B76" s="1" t="s">
         <v>76</v>
       </c>
-    </row>
-    <row r="77" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C76" t="s">
+        <v>357</v>
+      </c>
+    </row>
+    <row r="77" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A77">
         <v>76</v>
       </c>
       <c r="B77" s="1" t="s">
         <v>77</v>
       </c>
-    </row>
-    <row r="78" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C77" t="s">
+        <v>357</v>
+      </c>
+    </row>
+    <row r="78" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A78">
         <v>77</v>
       </c>
       <c r="B78" s="1" t="s">
         <v>78</v>
       </c>
-    </row>
-    <row r="79" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C78" t="s">
+        <v>357</v>
+      </c>
+    </row>
+    <row r="79" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A79">
         <v>78</v>
       </c>
       <c r="B79" s="1" t="s">
         <v>79</v>
       </c>
-    </row>
-    <row r="80" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C79" t="s">
+        <v>357</v>
+      </c>
+    </row>
+    <row r="80" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A80">
         <v>79</v>
       </c>
       <c r="B80" s="1" t="s">
         <v>80</v>
       </c>
-    </row>
-    <row r="81" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C80" t="s">
+        <v>357</v>
+      </c>
+    </row>
+    <row r="81" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A81">
         <v>80</v>
       </c>
       <c r="B81" s="1" t="s">
         <v>81</v>
       </c>
-    </row>
-    <row r="82" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C81" t="s">
+        <v>357</v>
+      </c>
+    </row>
+    <row r="82" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A82">
         <v>81</v>
       </c>
       <c r="B82" s="1" t="s">
         <v>82</v>
       </c>
-    </row>
-    <row r="83" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C82" t="s">
+        <v>357</v>
+      </c>
+    </row>
+    <row r="83" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A83">
         <v>82</v>
       </c>
       <c r="B83" s="1" t="s">
         <v>83</v>
       </c>
-    </row>
-    <row r="84" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C83" t="s">
+        <v>357</v>
+      </c>
+    </row>
+    <row r="84" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A84">
         <v>83</v>
       </c>
       <c r="B84" s="1" t="s">
         <v>84</v>
       </c>
-    </row>
-    <row r="85" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C84" t="s">
+        <v>357</v>
+      </c>
+    </row>
+    <row r="85" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A85">
         <v>84</v>
       </c>
       <c r="B85" s="1" t="s">
         <v>85</v>
       </c>
-    </row>
-    <row r="86" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C85" t="s">
+        <v>357</v>
+      </c>
+    </row>
+    <row r="86" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A86">
         <v>85</v>
       </c>
       <c r="B86" s="1" t="s">
         <v>86</v>
       </c>
-    </row>
-    <row r="87" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C86" t="s">
+        <v>357</v>
+      </c>
+    </row>
+    <row r="87" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A87">
         <v>86</v>
       </c>
       <c r="B87" s="1" t="s">
         <v>87</v>
       </c>
-    </row>
-    <row r="88" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C87" t="s">
+        <v>357</v>
+      </c>
+    </row>
+    <row r="88" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A88">
         <v>87</v>
       </c>
       <c r="B88" s="1" t="s">
         <v>88</v>
       </c>
-    </row>
-    <row r="89" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C88" t="s">
+        <v>357</v>
+      </c>
+    </row>
+    <row r="89" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A89">
         <v>88</v>
       </c>
       <c r="B89" s="1" t="s">
         <v>89</v>
       </c>
-    </row>
-    <row r="90" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C89" t="s">
+        <v>357</v>
+      </c>
+    </row>
+    <row r="90" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A90">
         <v>89</v>
       </c>
       <c r="B90" s="1" t="s">
         <v>90</v>
       </c>
-    </row>
-    <row r="91" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C90" t="s">
+        <v>357</v>
+      </c>
+    </row>
+    <row r="91" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A91">
         <v>90</v>
       </c>
       <c r="B91" s="1" t="s">
         <v>91</v>
       </c>
-    </row>
-    <row r="92" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C91" t="s">
+        <v>357</v>
+      </c>
+    </row>
+    <row r="92" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A92">
         <v>91</v>
       </c>
       <c r="B92" s="1" t="s">
         <v>92</v>
       </c>
-    </row>
-    <row r="93" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C92" t="s">
+        <v>357</v>
+      </c>
+    </row>
+    <row r="93" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A93">
         <v>92</v>
       </c>
       <c r="B93" s="1" t="s">
         <v>93</v>
       </c>
-    </row>
-    <row r="94" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C93" t="s">
+        <v>357</v>
+      </c>
+    </row>
+    <row r="94" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A94">
         <v>93</v>
       </c>
       <c r="B94" s="1" t="s">
         <v>94</v>
       </c>
-    </row>
-    <row r="95" spans="1:2" ht="30" x14ac:dyDescent="0.25">
+      <c r="C94" t="s">
+        <v>357</v>
+      </c>
+    </row>
+    <row r="95" spans="1:3" ht="30" x14ac:dyDescent="0.25">
       <c r="A95">
         <v>94</v>
       </c>
       <c r="B95" s="1" t="s">
         <v>95</v>
       </c>
-    </row>
-    <row r="96" spans="1:2" ht="30" x14ac:dyDescent="0.25">
+      <c r="C95" t="s">
+        <v>357</v>
+      </c>
+    </row>
+    <row r="96" spans="1:3" ht="30" x14ac:dyDescent="0.25">
       <c r="A96">
         <v>95</v>
       </c>
       <c r="B96" s="1" t="s">
         <v>96</v>
       </c>
-    </row>
-    <row r="97" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C96" t="s">
+        <v>357</v>
+      </c>
+    </row>
+    <row r="97" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A97">
         <v>96</v>
       </c>
       <c r="B97" s="1" t="s">
         <v>97</v>
       </c>
-    </row>
-    <row r="98" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C97" t="s">
+        <v>357</v>
+      </c>
+    </row>
+    <row r="98" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A98">
         <v>97</v>
       </c>
       <c r="B98" s="1" t="s">
         <v>98</v>
       </c>
-    </row>
-    <row r="99" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C98" t="s">
+        <v>357</v>
+      </c>
+    </row>
+    <row r="99" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A99">
         <v>98</v>
       </c>
       <c r="B99" s="1" t="s">
         <v>99</v>
       </c>
-    </row>
-    <row r="100" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C99" t="s">
+        <v>357</v>
+      </c>
+    </row>
+    <row r="100" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A100">
         <v>99</v>
       </c>
       <c r="B100" s="1" t="s">
         <v>100</v>
       </c>
-    </row>
-    <row r="101" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C100" t="s">
+        <v>357</v>
+      </c>
+    </row>
+    <row r="101" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A101">
         <v>100</v>
       </c>
       <c r="B101" s="1" t="s">
         <v>101</v>
       </c>
-    </row>
-    <row r="102" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C101" t="s">
+        <v>357</v>
+      </c>
+    </row>
+    <row r="102" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A102">
         <v>101</v>
       </c>
       <c r="B102" s="1" t="s">
         <v>102</v>
       </c>
-    </row>
-    <row r="103" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C102" t="s">
+        <v>357</v>
+      </c>
+    </row>
+    <row r="103" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A103">
         <v>102</v>
       </c>
       <c r="B103" s="1" t="s">
         <v>103</v>
       </c>
-    </row>
-    <row r="104" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C103" t="s">
+        <v>357</v>
+      </c>
+    </row>
+    <row r="104" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A104">
         <v>103</v>
       </c>
       <c r="B104" s="1" t="s">
         <v>104</v>
       </c>
-    </row>
-    <row r="105" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C104" t="s">
+        <v>357</v>
+      </c>
+    </row>
+    <row r="105" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A105">
         <v>104</v>
       </c>
       <c r="B105" s="1" t="s">
         <v>105</v>
       </c>
-    </row>
-    <row r="106" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C105" t="s">
+        <v>357</v>
+      </c>
+    </row>
+    <row r="106" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A106">
         <v>105</v>
       </c>
       <c r="B106" s="1" t="s">
         <v>106</v>
       </c>
-    </row>
-    <row r="107" spans="1:2" ht="30" x14ac:dyDescent="0.25">
+      <c r="C106" t="s">
+        <v>357</v>
+      </c>
+    </row>
+    <row r="107" spans="1:3" ht="30" x14ac:dyDescent="0.25">
       <c r="A107">
         <v>106</v>
       </c>
       <c r="B107" s="1" t="s">
         <v>107</v>
       </c>
-    </row>
-    <row r="108" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C107" t="s">
+        <v>357</v>
+      </c>
+    </row>
+    <row r="108" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A108">
         <v>107</v>
       </c>
       <c r="B108" s="1" t="s">
         <v>108</v>
       </c>
-    </row>
-    <row r="109" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C108" t="s">
+        <v>357</v>
+      </c>
+    </row>
+    <row r="109" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A109">
         <v>108</v>
       </c>
       <c r="B109" s="1" t="s">
         <v>109</v>
       </c>
-    </row>
-    <row r="110" spans="1:2" ht="45" x14ac:dyDescent="0.25">
+      <c r="C109" t="s">
+        <v>357</v>
+      </c>
+    </row>
+    <row r="110" spans="1:3" ht="45" x14ac:dyDescent="0.25">
       <c r="A110">
         <v>109</v>
       </c>
       <c r="B110" s="1" t="s">
         <v>110</v>
       </c>
-    </row>
-    <row r="111" spans="1:2" ht="45" x14ac:dyDescent="0.25">
+      <c r="C110" t="s">
+        <v>357</v>
+      </c>
+    </row>
+    <row r="111" spans="1:3" ht="45" x14ac:dyDescent="0.25">
       <c r="A111">
         <v>110</v>
       </c>
       <c r="B111" s="1" t="s">
         <v>111</v>
       </c>
-    </row>
-    <row r="112" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C111" t="s">
+        <v>357</v>
+      </c>
+    </row>
+    <row r="112" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A112">
         <v>111</v>
       </c>
       <c r="B112" s="1" t="s">
         <v>112</v>
       </c>
-    </row>
-    <row r="113" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C112" t="s">
+        <v>357</v>
+      </c>
+    </row>
+    <row r="113" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A113">
         <v>112</v>
       </c>
       <c r="B113" s="1" t="s">
         <v>113</v>
       </c>
-    </row>
-    <row r="114" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C113" t="s">
+        <v>357</v>
+      </c>
+    </row>
+    <row r="114" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A114">
         <v>113</v>
       </c>
       <c r="B114" s="1" t="s">
         <v>114</v>
       </c>
-    </row>
-    <row r="115" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C114" t="s">
+        <v>357</v>
+      </c>
+    </row>
+    <row r="115" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A115">
         <v>114</v>
       </c>
       <c r="B115" s="1" t="s">
         <v>115</v>
       </c>
-    </row>
-    <row r="116" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C115" t="s">
+        <v>357</v>
+      </c>
+    </row>
+    <row r="116" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A116">
         <v>115</v>
       </c>
       <c r="B116" s="1" t="s">
         <v>116</v>
       </c>
-    </row>
-    <row r="117" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C116" t="s">
+        <v>357</v>
+      </c>
+    </row>
+    <row r="117" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A117">
         <v>116</v>
       </c>
       <c r="B117" s="1" t="s">
         <v>117</v>
       </c>
-    </row>
-    <row r="118" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C117" t="s">
+        <v>357</v>
+      </c>
+    </row>
+    <row r="118" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A118">
         <v>117</v>
       </c>
       <c r="B118" s="1" t="s">
         <v>118</v>
       </c>
-    </row>
-    <row r="119" spans="1:2" ht="30" x14ac:dyDescent="0.25">
+      <c r="C118" t="s">
+        <v>357</v>
+      </c>
+    </row>
+    <row r="119" spans="1:3" ht="30" x14ac:dyDescent="0.25">
       <c r="A119">
         <v>118</v>
       </c>
       <c r="B119" s="1" t="s">
         <v>119</v>
       </c>
-    </row>
-    <row r="120" spans="1:2" ht="45" x14ac:dyDescent="0.25">
+      <c r="C119" t="s">
+        <v>357</v>
+      </c>
+    </row>
+    <row r="120" spans="1:3" ht="45" x14ac:dyDescent="0.25">
       <c r="A120">
         <v>119</v>
       </c>
       <c r="B120" s="1" t="s">
         <v>120</v>
       </c>
-    </row>
-    <row r="121" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C120" t="s">
+        <v>357</v>
+      </c>
+    </row>
+    <row r="121" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A121">
         <v>120</v>
       </c>
       <c r="B121" s="1" t="s">
         <v>121</v>
       </c>
-    </row>
-    <row r="122" spans="1:2" ht="30" x14ac:dyDescent="0.25">
+      <c r="C121" t="s">
+        <v>357</v>
+      </c>
+    </row>
+    <row r="122" spans="1:3" ht="30" x14ac:dyDescent="0.25">
       <c r="A122">
         <v>121</v>
       </c>
       <c r="B122" s="1" t="s">
         <v>122</v>
       </c>
-    </row>
-    <row r="123" spans="1:2" ht="90" x14ac:dyDescent="0.25">
+      <c r="C122" t="s">
+        <v>357</v>
+      </c>
+    </row>
+    <row r="123" spans="1:3" ht="90" x14ac:dyDescent="0.25">
       <c r="A123">
         <v>122</v>
       </c>
       <c r="B123" s="1" t="s">
         <v>123</v>
       </c>
-    </row>
-    <row r="124" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C123" t="s">
+        <v>357</v>
+      </c>
+    </row>
+    <row r="124" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A124">
         <v>123</v>
       </c>
       <c r="B124" s="1" t="s">
         <v>124</v>
       </c>
-    </row>
-    <row r="125" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C124" t="s">
+        <v>357</v>
+      </c>
+    </row>
+    <row r="125" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A125">
         <v>124</v>
       </c>
       <c r="B125" s="1" t="s">
         <v>125</v>
       </c>
-    </row>
-    <row r="126" spans="1:2" ht="30" x14ac:dyDescent="0.25">
+      <c r="C125" t="s">
+        <v>357</v>
+      </c>
+    </row>
+    <row r="126" spans="1:3" ht="30" x14ac:dyDescent="0.25">
       <c r="A126">
         <v>125</v>
       </c>
       <c r="B126" s="1" t="s">
         <v>126</v>
       </c>
-    </row>
-    <row r="127" spans="1:2" ht="30" x14ac:dyDescent="0.25">
+      <c r="C126" t="s">
+        <v>357</v>
+      </c>
+    </row>
+    <row r="127" spans="1:3" ht="30" x14ac:dyDescent="0.25">
       <c r="A127">
         <v>126</v>
       </c>
       <c r="B127" s="1" t="s">
         <v>127</v>
       </c>
-    </row>
-    <row r="128" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C127" t="s">
+        <v>357</v>
+      </c>
+    </row>
+    <row r="128" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A128">
         <v>127</v>
       </c>
       <c r="B128" s="1" t="s">
         <v>128</v>
       </c>
-    </row>
-    <row r="129" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C128" t="s">
+        <v>357</v>
+      </c>
+    </row>
+    <row r="129" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A129">
         <v>128</v>
       </c>
       <c r="B129" s="1" t="s">
         <v>129</v>
       </c>
-    </row>
-    <row r="130" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C129" t="s">
+        <v>357</v>
+      </c>
+    </row>
+    <row r="130" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A130">
         <v>129</v>
       </c>
       <c r="B130" s="1" t="s">
         <v>130</v>
       </c>
-    </row>
-    <row r="131" spans="1:2" ht="45" x14ac:dyDescent="0.25">
+      <c r="C130" t="s">
+        <v>357</v>
+      </c>
+    </row>
+    <row r="131" spans="1:3" ht="45" x14ac:dyDescent="0.25">
       <c r="A131">
         <v>130</v>
       </c>
       <c r="B131" s="1" t="s">
         <v>131</v>
       </c>
-    </row>
-    <row r="132" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C131" t="s">
+        <v>357</v>
+      </c>
+    </row>
+    <row r="132" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A132">
         <v>131</v>
       </c>
       <c r="B132" s="1" t="s">
         <v>132</v>
       </c>
-    </row>
-    <row r="133" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C132" t="s">
+        <v>357</v>
+      </c>
+    </row>
+    <row r="133" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A133">
         <v>132</v>
       </c>
       <c r="B133" s="1" t="s">
         <v>133</v>
       </c>
-    </row>
-    <row r="134" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C133" t="s">
+        <v>357</v>
+      </c>
+    </row>
+    <row r="134" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A134">
         <v>133</v>
       </c>
       <c r="B134" s="1" t="s">
         <v>134</v>
       </c>
-    </row>
-    <row r="135" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C134" t="s">
+        <v>357</v>
+      </c>
+    </row>
+    <row r="135" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A135">
         <v>134</v>
       </c>
       <c r="B135" s="1" t="s">
         <v>135</v>
       </c>
-    </row>
-    <row r="136" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C135" t="s">
+        <v>357</v>
+      </c>
+    </row>
+    <row r="136" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A136">
         <v>135</v>
       </c>
       <c r="B136" s="1" t="s">
         <v>136</v>
       </c>
-    </row>
-    <row r="137" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C136" t="s">
+        <v>357</v>
+      </c>
+    </row>
+    <row r="137" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A137">
         <v>136</v>
       </c>
       <c r="B137" s="1" t="s">
         <v>137</v>
       </c>
-    </row>
-    <row r="138" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C137" t="s">
+        <v>357</v>
+      </c>
+    </row>
+    <row r="138" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A138">
         <v>137</v>
       </c>
       <c r="B138" s="1" t="s">
         <v>138</v>
       </c>
-    </row>
-    <row r="139" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C138" t="s">
+        <v>357</v>
+      </c>
+    </row>
+    <row r="139" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A139">
         <v>138</v>
       </c>
       <c r="B139" s="1" t="s">
         <v>139</v>
       </c>
-    </row>
-    <row r="140" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C139" t="s">
+        <v>357</v>
+      </c>
+    </row>
+    <row r="140" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A140">
         <v>139</v>
       </c>
       <c r="B140" s="1" t="s">
         <v>140</v>
       </c>
-    </row>
-    <row r="141" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C140" t="s">
+        <v>357</v>
+      </c>
+    </row>
+    <row r="141" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A141">
         <v>140</v>
       </c>
       <c r="B141" s="1" t="s">
         <v>141</v>
       </c>
-    </row>
-    <row r="142" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C141" t="s">
+        <v>358</v>
+      </c>
+    </row>
+    <row r="142" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A142">
         <v>141</v>
       </c>
       <c r="B142" s="1" t="s">
         <v>142</v>
       </c>
-    </row>
-    <row r="143" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C142" t="s">
+        <v>358</v>
+      </c>
+    </row>
+    <row r="143" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A143">
         <v>142</v>
       </c>
       <c r="B143" s="1" t="s">
         <v>143</v>
       </c>
-    </row>
-    <row r="144" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C143" t="s">
+        <v>358</v>
+      </c>
+    </row>
+    <row r="144" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A144">
         <v>143</v>
       </c>
       <c r="B144" s="1" t="s">
         <v>144</v>
       </c>
-    </row>
-    <row r="145" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C144" t="s">
+        <v>358</v>
+      </c>
+    </row>
+    <row r="145" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A145">
         <v>144</v>
       </c>
       <c r="B145" s="1" t="s">
         <v>145</v>
       </c>
-    </row>
-    <row r="146" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C145" t="s">
+        <v>357</v>
+      </c>
+    </row>
+    <row r="146" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A146">
         <v>145</v>
       </c>
       <c r="B146" s="1" t="s">
         <v>146</v>
       </c>
-    </row>
-    <row r="147" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C146" t="s">
+        <v>357</v>
+      </c>
+    </row>
+    <row r="147" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A147">
         <v>146</v>
       </c>
       <c r="B147" s="1" t="s">
         <v>147</v>
       </c>
-    </row>
-    <row r="148" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C147" t="s">
+        <v>357</v>
+      </c>
+    </row>
+    <row r="148" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A148">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="B148" s="1" t="s">
         <v>148</v>
       </c>
-    </row>
-    <row r="149" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C148" t="s">
+        <v>359</v>
+      </c>
+    </row>
+    <row r="149" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A149">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="B149" s="1" t="s">
         <v>149</v>
       </c>
-    </row>
-    <row r="150" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C149" t="s">
+        <v>359</v>
+      </c>
+    </row>
+    <row r="150" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A150">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="B150" s="1" t="s">
         <v>150</v>
       </c>
-    </row>
-    <row r="151" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C150" t="s">
+        <v>359</v>
+      </c>
+    </row>
+    <row r="151" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A151">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="B151" s="1" t="s">
         <v>151</v>
       </c>
-    </row>
-    <row r="152" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C151" t="s">
+        <v>359</v>
+      </c>
+    </row>
+    <row r="152" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A152">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="B152" s="1" t="s">
         <v>152</v>
       </c>
-    </row>
-    <row r="153" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C152" t="s">
+        <v>359</v>
+      </c>
+    </row>
+    <row r="153" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A153">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="B153" s="1" t="s">
         <v>153</v>
       </c>
-    </row>
-    <row r="154" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C153" t="s">
+        <v>359</v>
+      </c>
+    </row>
+    <row r="154" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A154">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="B154" s="1" t="s">
         <v>154</v>
       </c>
-    </row>
-    <row r="155" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C154" t="s">
+        <v>359</v>
+      </c>
+    </row>
+    <row r="155" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A155">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="B155" s="1" t="s">
         <v>155</v>
       </c>
-    </row>
-    <row r="156" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C155" t="s">
+        <v>359</v>
+      </c>
+    </row>
+    <row r="156" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A156">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="B156" s="1" t="s">
         <v>156</v>
       </c>
-    </row>
-    <row r="157" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C156" t="s">
+        <v>357</v>
+      </c>
+    </row>
+    <row r="157" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A157">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="B157" s="1" t="s">
         <v>157</v>
       </c>
-    </row>
-    <row r="158" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C157" t="s">
+        <v>359</v>
+      </c>
+    </row>
+    <row r="158" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A158">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="B158" s="1" t="s">
         <v>158</v>
       </c>
-    </row>
-    <row r="159" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C158" t="s">
+        <v>357</v>
+      </c>
+    </row>
+    <row r="159" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A159">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="B159" s="1" t="s">
         <v>159</v>
       </c>
-    </row>
-    <row r="160" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C159" t="s">
+        <v>359</v>
+      </c>
+    </row>
+    <row r="160" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A160">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="B160" s="1" t="s">
         <v>160</v>
       </c>
+      <c r="C160" t="s">
+        <v>357</v>
+      </c>
     </row>
     <row r="161" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A161">
-        <v>160</v>
+        <v>518</v>
       </c>
       <c r="B161" s="1" t="s">
         <v>161</v>
       </c>
+      <c r="C161" t="s">
+        <v>357</v>
+      </c>
     </row>
     <row r="162" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A162">
-        <v>518</v>
+        <v>519</v>
       </c>
       <c r="B162" s="1" t="s">
         <v>162</v>
       </c>
       <c r="C162" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
     </row>
     <row r="163" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A163">
-        <v>519</v>
+        <v>520</v>
       </c>
       <c r="B163" s="1" t="s">
         <v>163</v>
       </c>
       <c r="C163" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
     </row>
     <row r="164" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A164">
-        <v>520</v>
+        <v>521</v>
       </c>
       <c r="B164" s="1" t="s">
         <v>164</v>
       </c>
       <c r="C164" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
     </row>
     <row r="165" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A165">
-        <v>521</v>
+        <v>522</v>
       </c>
       <c r="B165" s="1" t="s">
         <v>165</v>
       </c>
       <c r="C165" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
     </row>
     <row r="166" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A166">
-        <v>522</v>
+        <v>523</v>
       </c>
       <c r="B166" s="1" t="s">
         <v>166</v>
       </c>
       <c r="C166" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
     </row>
     <row r="167" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A167">
-        <v>523</v>
+        <v>524</v>
       </c>
       <c r="B167" s="1" t="s">
         <v>167</v>
       </c>
       <c r="C167" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
     </row>
     <row r="168" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A168">
-        <v>524</v>
+        <v>525</v>
       </c>
       <c r="B168" s="1" t="s">
         <v>168</v>
       </c>
       <c r="C168" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
     </row>
     <row r="169" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A169">
-        <v>525</v>
+        <v>526</v>
       </c>
       <c r="B169" s="1" t="s">
         <v>169</v>
       </c>
       <c r="C169" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
     </row>
     <row r="170" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A170">
-        <v>526</v>
+        <v>527</v>
       </c>
       <c r="B170" s="1" t="s">
         <v>170</v>
       </c>
       <c r="C170" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
     </row>
     <row r="171" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A171">
-        <v>527</v>
+        <v>528</v>
       </c>
       <c r="B171" s="1" t="s">
         <v>171</v>
       </c>
       <c r="C171" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
     </row>
     <row r="172" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A172">
-        <v>528</v>
+        <v>529</v>
       </c>
       <c r="B172" s="1" t="s">
         <v>172</v>
       </c>
       <c r="C172" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
     </row>
     <row r="173" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A173">
-        <v>529</v>
+        <v>530</v>
       </c>
       <c r="B173" s="1" t="s">
         <v>173</v>
       </c>
       <c r="C173" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
     </row>
     <row r="174" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A174">
-        <v>530</v>
+        <v>531</v>
       </c>
       <c r="B174" s="1" t="s">
         <v>174</v>
       </c>
       <c r="C174" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
     </row>
     <row r="175" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A175">
-        <v>531</v>
+        <v>532</v>
       </c>
       <c r="B175" s="1" t="s">
         <v>175</v>
       </c>
       <c r="C175" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
     </row>
     <row r="176" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A176">
-        <v>532</v>
+        <v>533</v>
       </c>
       <c r="B176" s="1" t="s">
         <v>176</v>
       </c>
       <c r="C176" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
     </row>
     <row r="177" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A177">
-        <v>533</v>
+        <v>534</v>
       </c>
       <c r="B177" s="1" t="s">
         <v>177</v>
       </c>
       <c r="C177" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
     </row>
     <row r="178" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A178">
-        <v>534</v>
+        <v>535</v>
       </c>
       <c r="B178" s="1" t="s">
         <v>178</v>
@@ -2990,502 +3467,502 @@
     </row>
     <row r="179" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A179">
-        <v>535</v>
+        <v>536</v>
       </c>
       <c r="B179" s="1" t="s">
         <v>179</v>
       </c>
       <c r="C179" t="s">
-        <v>360</v>
+        <v>359</v>
       </c>
     </row>
     <row r="180" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A180">
-        <v>536</v>
+        <v>537</v>
       </c>
       <c r="B180" s="1" t="s">
         <v>180</v>
       </c>
       <c r="C180" t="s">
-        <v>360</v>
+        <v>357</v>
       </c>
     </row>
     <row r="181" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A181">
-        <v>537</v>
+        <v>538</v>
       </c>
       <c r="B181" s="1" t="s">
         <v>181</v>
       </c>
       <c r="C181" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
     </row>
     <row r="182" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A182">
-        <v>538</v>
+        <v>539</v>
       </c>
       <c r="B182" s="1" t="s">
         <v>182</v>
       </c>
       <c r="C182" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
     </row>
     <row r="183" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A183">
-        <v>539</v>
+        <v>540</v>
       </c>
       <c r="B183" s="1" t="s">
         <v>183</v>
       </c>
       <c r="C183" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
     </row>
     <row r="184" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A184">
-        <v>540</v>
+        <v>541</v>
       </c>
       <c r="B184" s="1" t="s">
         <v>184</v>
       </c>
       <c r="C184" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
     </row>
     <row r="185" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A185">
-        <v>541</v>
+        <v>542</v>
       </c>
       <c r="B185" s="1" t="s">
         <v>185</v>
       </c>
       <c r="C185" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
     </row>
     <row r="186" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A186">
-        <v>542</v>
+        <v>543</v>
       </c>
       <c r="B186" s="1" t="s">
         <v>186</v>
       </c>
       <c r="C186" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
     </row>
     <row r="187" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A187">
-        <v>543</v>
+        <v>544</v>
       </c>
       <c r="B187" s="1" t="s">
         <v>187</v>
       </c>
       <c r="C187" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
     </row>
     <row r="188" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A188">
-        <v>544</v>
+        <v>545</v>
       </c>
       <c r="B188" s="1" t="s">
         <v>188</v>
       </c>
       <c r="C188" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
     </row>
     <row r="189" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A189">
-        <v>545</v>
+        <v>546</v>
       </c>
       <c r="B189" s="1" t="s">
         <v>189</v>
       </c>
       <c r="C189" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
     </row>
     <row r="190" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A190">
-        <v>546</v>
+        <v>547</v>
       </c>
       <c r="B190" s="1" t="s">
         <v>190</v>
       </c>
       <c r="C190" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
     </row>
     <row r="191" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A191">
-        <v>547</v>
+        <v>548</v>
       </c>
       <c r="B191" s="1" t="s">
         <v>191</v>
       </c>
       <c r="C191" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
     </row>
     <row r="192" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A192">
-        <v>548</v>
+        <v>549</v>
       </c>
       <c r="B192" s="1" t="s">
         <v>192</v>
       </c>
       <c r="C192" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
     </row>
     <row r="193" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A193">
-        <v>549</v>
+        <v>550</v>
       </c>
       <c r="B193" s="1" t="s">
         <v>193</v>
       </c>
       <c r="C193" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
     </row>
     <row r="194" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A194">
-        <v>550</v>
+        <v>551</v>
       </c>
       <c r="B194" s="1" t="s">
         <v>194</v>
       </c>
       <c r="C194" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
     </row>
     <row r="195" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A195">
-        <v>551</v>
+        <v>552</v>
       </c>
       <c r="B195" s="1" t="s">
         <v>195</v>
       </c>
       <c r="C195" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
     </row>
     <row r="196" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A196">
-        <v>552</v>
+        <v>553</v>
       </c>
       <c r="B196" s="1" t="s">
         <v>196</v>
       </c>
       <c r="C196" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
     </row>
     <row r="197" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A197">
-        <v>553</v>
+        <v>554</v>
       </c>
       <c r="B197" s="1" t="s">
         <v>197</v>
       </c>
       <c r="C197" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
     </row>
     <row r="198" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A198">
-        <v>554</v>
+        <v>555</v>
       </c>
       <c r="B198" s="1" t="s">
         <v>198</v>
       </c>
       <c r="C198" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
     </row>
     <row r="199" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A199">
-        <v>555</v>
+        <v>556</v>
       </c>
       <c r="B199" s="1" t="s">
         <v>199</v>
       </c>
       <c r="C199" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
     </row>
     <row r="200" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A200">
-        <v>556</v>
+        <v>557</v>
       </c>
       <c r="B200" s="1" t="s">
         <v>200</v>
       </c>
       <c r="C200" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
     </row>
     <row r="201" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A201">
-        <v>557</v>
+        <v>558</v>
       </c>
       <c r="B201" s="1" t="s">
         <v>201</v>
       </c>
       <c r="C201" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
     </row>
     <row r="202" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A202">
-        <v>558</v>
+        <v>559</v>
       </c>
       <c r="B202" s="1" t="s">
         <v>202</v>
       </c>
       <c r="C202" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
     </row>
     <row r="203" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A203">
-        <v>559</v>
+        <v>560</v>
       </c>
       <c r="B203" s="1" t="s">
         <v>203</v>
       </c>
       <c r="C203" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
     </row>
     <row r="204" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A204">
-        <v>560</v>
+        <v>561</v>
       </c>
       <c r="B204" s="1" t="s">
         <v>204</v>
       </c>
       <c r="C204" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
     </row>
     <row r="205" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A205">
-        <v>561</v>
+        <v>562</v>
       </c>
       <c r="B205" s="1" t="s">
         <v>205</v>
       </c>
       <c r="C205" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
     </row>
     <row r="206" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A206">
-        <v>562</v>
+        <v>563</v>
       </c>
       <c r="B206" s="1" t="s">
         <v>206</v>
       </c>
       <c r="C206" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
     </row>
     <row r="207" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A207">
-        <v>563</v>
+        <v>564</v>
       </c>
       <c r="B207" s="1" t="s">
         <v>207</v>
       </c>
       <c r="C207" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
     </row>
     <row r="208" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A208">
-        <v>564</v>
+        <v>565</v>
       </c>
       <c r="B208" s="1" t="s">
         <v>208</v>
       </c>
       <c r="C208" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
     </row>
     <row r="209" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A209">
-        <v>565</v>
+        <v>566</v>
       </c>
       <c r="B209" s="1" t="s">
         <v>209</v>
       </c>
       <c r="C209" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
     </row>
     <row r="210" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A210">
-        <v>566</v>
+        <v>567</v>
       </c>
       <c r="B210" s="1" t="s">
         <v>210</v>
       </c>
       <c r="C210" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
     </row>
     <row r="211" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A211">
-        <v>567</v>
+        <v>568</v>
       </c>
       <c r="B211" s="1" t="s">
         <v>211</v>
       </c>
       <c r="C211" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
     </row>
     <row r="212" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A212">
-        <v>568</v>
+        <v>569</v>
       </c>
       <c r="B212" s="1" t="s">
         <v>212</v>
       </c>
       <c r="C212" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
     </row>
     <row r="213" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A213">
-        <v>569</v>
+        <v>570</v>
       </c>
       <c r="B213" s="1" t="s">
         <v>213</v>
       </c>
       <c r="C213" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
     </row>
     <row r="214" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A214">
-        <v>570</v>
+        <v>571</v>
       </c>
       <c r="B214" s="1" t="s">
         <v>214</v>
       </c>
       <c r="C214" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
     </row>
     <row r="215" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A215">
-        <v>571</v>
+        <v>572</v>
       </c>
       <c r="B215" s="1" t="s">
         <v>215</v>
       </c>
       <c r="C215" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
     </row>
     <row r="216" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A216">
-        <v>572</v>
+        <v>573</v>
       </c>
       <c r="B216" s="1" t="s">
         <v>216</v>
       </c>
       <c r="C216" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
     </row>
     <row r="217" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A217">
-        <v>573</v>
+        <v>574</v>
       </c>
       <c r="B217" s="1" t="s">
         <v>217</v>
       </c>
       <c r="C217" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
     </row>
     <row r="218" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A218">
-        <v>574</v>
+        <v>575</v>
       </c>
       <c r="B218" s="1" t="s">
         <v>218</v>
       </c>
       <c r="C218" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
     </row>
     <row r="219" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A219">
-        <v>575</v>
+        <v>576</v>
       </c>
       <c r="B219" s="1" t="s">
         <v>219</v>
       </c>
       <c r="C219" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
     </row>
     <row r="220" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A220">
-        <v>576</v>
+        <v>577</v>
       </c>
       <c r="B220" s="1" t="s">
         <v>220</v>
       </c>
       <c r="C220" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
     </row>
     <row r="221" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A221">
-        <v>577</v>
+        <v>578</v>
       </c>
       <c r="B221" s="1" t="s">
         <v>221</v>
       </c>
       <c r="C221" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
     </row>
     <row r="222" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A222">
-        <v>578</v>
+        <v>579</v>
       </c>
       <c r="B222" s="1" t="s">
         <v>222</v>
       </c>
       <c r="C222" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
     </row>
     <row r="223" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A223">
-        <v>579</v>
+        <v>580</v>
       </c>
       <c r="B223" s="1" t="s">
         <v>223</v>
       </c>
       <c r="C223" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
     </row>
     <row r="224" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A224">
-        <v>580</v>
+        <v>581</v>
       </c>
       <c r="B224" s="1" t="s">
         <v>224</v>
@@ -3496,1468 +3973,1458 @@
     </row>
     <row r="225" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A225">
-        <v>581</v>
+        <v>582</v>
       </c>
       <c r="B225" s="1" t="s">
         <v>225</v>
       </c>
       <c r="C225" t="s">
-        <v>360</v>
+        <v>359</v>
       </c>
     </row>
     <row r="226" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A226">
-        <v>582</v>
+        <v>583</v>
       </c>
       <c r="B226" s="1" t="s">
         <v>226</v>
       </c>
       <c r="C226" t="s">
-        <v>360</v>
+        <v>359</v>
       </c>
     </row>
     <row r="227" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A227">
-        <v>583</v>
+        <v>584</v>
       </c>
       <c r="B227" s="1" t="s">
         <v>227</v>
       </c>
       <c r="C227" t="s">
-        <v>360</v>
+        <v>359</v>
       </c>
     </row>
     <row r="228" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A228">
-        <v>584</v>
+        <v>585</v>
       </c>
       <c r="B228" s="1" t="s">
         <v>228</v>
       </c>
       <c r="C228" t="s">
-        <v>360</v>
+        <v>359</v>
       </c>
     </row>
     <row r="229" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A229">
-        <v>585</v>
+        <v>586</v>
       </c>
       <c r="B229" s="1" t="s">
         <v>229</v>
       </c>
       <c r="C229" t="s">
-        <v>360</v>
+        <v>359</v>
       </c>
     </row>
     <row r="230" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A230">
-        <v>586</v>
+        <v>587</v>
       </c>
       <c r="B230" s="1" t="s">
         <v>230</v>
       </c>
       <c r="C230" t="s">
-        <v>360</v>
+        <v>359</v>
       </c>
     </row>
     <row r="231" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A231">
-        <v>587</v>
+        <v>588</v>
       </c>
       <c r="B231" s="1" t="s">
         <v>231</v>
       </c>
       <c r="C231" t="s">
-        <v>360</v>
+        <v>359</v>
       </c>
     </row>
     <row r="232" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A232">
-        <v>588</v>
+        <v>589</v>
       </c>
       <c r="B232" s="1" t="s">
         <v>232</v>
       </c>
       <c r="C232" t="s">
-        <v>360</v>
+        <v>359</v>
       </c>
     </row>
     <row r="233" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A233">
-        <v>589</v>
+        <v>590</v>
       </c>
       <c r="B233" s="1" t="s">
         <v>233</v>
       </c>
       <c r="C233" t="s">
-        <v>360</v>
+        <v>359</v>
       </c>
     </row>
     <row r="234" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A234">
-        <v>590</v>
+        <v>591</v>
       </c>
       <c r="B234" s="1" t="s">
         <v>234</v>
       </c>
       <c r="C234" t="s">
-        <v>360</v>
+        <v>357</v>
       </c>
     </row>
     <row r="235" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A235">
-        <v>591</v>
+        <v>592</v>
       </c>
       <c r="B235" s="1" t="s">
         <v>235</v>
       </c>
       <c r="C235" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
     </row>
     <row r="236" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A236">
-        <v>592</v>
+        <v>593</v>
       </c>
       <c r="B236" s="1" t="s">
         <v>236</v>
       </c>
       <c r="C236" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
     </row>
     <row r="237" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A237">
-        <v>593</v>
+        <v>594</v>
       </c>
       <c r="B237" s="1" t="s">
         <v>237</v>
       </c>
       <c r="C237" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
     </row>
     <row r="238" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A238">
-        <v>594</v>
+        <v>595</v>
       </c>
       <c r="B238" s="1" t="s">
         <v>238</v>
       </c>
       <c r="C238" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
     </row>
     <row r="239" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A239">
-        <v>595</v>
+        <v>596</v>
       </c>
       <c r="B239" s="1" t="s">
         <v>239</v>
       </c>
       <c r="C239" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
     </row>
     <row r="240" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A240">
-        <v>596</v>
+        <v>597</v>
       </c>
       <c r="B240" s="1" t="s">
         <v>240</v>
       </c>
       <c r="C240" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
     </row>
     <row r="241" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A241">
-        <v>597</v>
+        <v>598</v>
       </c>
       <c r="B241" s="1" t="s">
         <v>241</v>
       </c>
       <c r="C241" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
     </row>
     <row r="242" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A242">
-        <v>598</v>
+        <v>599</v>
       </c>
       <c r="B242" s="1" t="s">
         <v>242</v>
       </c>
       <c r="C242" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
     </row>
     <row r="243" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A243">
-        <v>599</v>
+        <v>600</v>
       </c>
       <c r="B243" s="1" t="s">
         <v>243</v>
       </c>
       <c r="C243" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
     </row>
     <row r="244" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A244">
-        <v>600</v>
+        <v>601</v>
       </c>
       <c r="B244" s="1" t="s">
         <v>244</v>
       </c>
       <c r="C244" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
     </row>
     <row r="245" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A245">
-        <v>601</v>
+        <v>602</v>
       </c>
       <c r="B245" s="1" t="s">
         <v>245</v>
       </c>
       <c r="C245" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
     </row>
     <row r="246" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A246">
-        <v>602</v>
+        <v>603</v>
       </c>
       <c r="B246" s="1" t="s">
         <v>246</v>
       </c>
       <c r="C246" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
     </row>
     <row r="247" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A247">
-        <v>603</v>
+        <v>604</v>
       </c>
       <c r="B247" s="1" t="s">
         <v>247</v>
       </c>
       <c r="C247" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
     </row>
     <row r="248" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A248">
-        <v>604</v>
+        <v>605</v>
       </c>
       <c r="B248" s="1" t="s">
         <v>248</v>
       </c>
       <c r="C248" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
     </row>
     <row r="249" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A249">
-        <v>605</v>
+        <v>606</v>
       </c>
       <c r="B249" s="1" t="s">
         <v>249</v>
       </c>
       <c r="C249" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
     </row>
     <row r="250" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A250">
-        <v>606</v>
+        <v>607</v>
       </c>
       <c r="B250" s="1" t="s">
         <v>250</v>
       </c>
       <c r="C250" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
     </row>
     <row r="251" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A251">
-        <v>607</v>
+        <v>608</v>
       </c>
       <c r="B251" s="1" t="s">
         <v>251</v>
       </c>
       <c r="C251" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
     </row>
     <row r="252" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A252">
-        <v>608</v>
+        <v>609</v>
       </c>
       <c r="B252" s="1" t="s">
         <v>252</v>
       </c>
       <c r="C252" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
     </row>
     <row r="253" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A253">
-        <v>609</v>
+        <v>610</v>
       </c>
       <c r="B253" s="1" t="s">
         <v>253</v>
       </c>
       <c r="C253" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
     </row>
     <row r="254" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A254">
-        <v>610</v>
+        <v>611</v>
       </c>
       <c r="B254" s="1" t="s">
         <v>254</v>
       </c>
       <c r="C254" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
     </row>
     <row r="255" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A255">
-        <v>611</v>
+        <v>612</v>
       </c>
       <c r="B255" s="1" t="s">
         <v>255</v>
       </c>
       <c r="C255" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
     </row>
     <row r="256" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A256">
-        <v>612</v>
+        <v>613</v>
       </c>
       <c r="B256" s="1" t="s">
         <v>256</v>
       </c>
       <c r="C256" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
     </row>
     <row r="257" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A257">
-        <v>613</v>
+        <v>614</v>
       </c>
       <c r="B257" s="1" t="s">
         <v>257</v>
       </c>
       <c r="C257" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
     </row>
     <row r="258" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A258">
-        <v>614</v>
+        <v>615</v>
       </c>
       <c r="B258" s="1" t="s">
         <v>258</v>
       </c>
       <c r="C258" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
     </row>
     <row r="259" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A259">
-        <v>615</v>
+        <v>616</v>
       </c>
       <c r="B259" s="1" t="s">
         <v>259</v>
       </c>
       <c r="C259" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
     </row>
     <row r="260" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A260">
-        <v>616</v>
+        <v>617</v>
       </c>
       <c r="B260" s="1" t="s">
         <v>260</v>
       </c>
       <c r="C260" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
     </row>
     <row r="261" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A261">
-        <v>617</v>
+        <v>618</v>
       </c>
       <c r="B261" s="1" t="s">
         <v>261</v>
       </c>
       <c r="C261" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
     </row>
     <row r="262" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A262">
-        <v>618</v>
+        <v>619</v>
       </c>
       <c r="B262" s="1" t="s">
         <v>262</v>
       </c>
       <c r="C262" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
     </row>
     <row r="263" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A263">
-        <v>619</v>
+        <v>620</v>
       </c>
       <c r="B263" s="1" t="s">
         <v>263</v>
       </c>
       <c r="C263" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
     </row>
     <row r="264" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A264">
-        <v>620</v>
+        <v>621</v>
       </c>
       <c r="B264" s="1" t="s">
         <v>264</v>
       </c>
       <c r="C264" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
     </row>
     <row r="265" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A265">
-        <v>621</v>
+        <v>622</v>
       </c>
       <c r="B265" s="1" t="s">
         <v>265</v>
       </c>
       <c r="C265" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
     </row>
     <row r="266" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A266">
-        <v>622</v>
+        <v>623</v>
       </c>
       <c r="B266" s="1" t="s">
         <v>266</v>
       </c>
       <c r="C266" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
     </row>
     <row r="267" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A267">
-        <v>623</v>
+        <v>624</v>
       </c>
       <c r="B267" s="1" t="s">
         <v>267</v>
       </c>
       <c r="C267" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
     </row>
     <row r="268" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A268">
-        <v>624</v>
+        <v>625</v>
       </c>
       <c r="B268" s="1" t="s">
         <v>268</v>
       </c>
       <c r="C268" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
     </row>
     <row r="269" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A269">
-        <v>625</v>
+        <v>626</v>
       </c>
       <c r="B269" s="1" t="s">
         <v>269</v>
       </c>
       <c r="C269" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
     </row>
     <row r="270" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A270">
-        <v>626</v>
+        <v>627</v>
       </c>
       <c r="B270" s="1" t="s">
         <v>270</v>
       </c>
       <c r="C270" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
     </row>
     <row r="271" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A271">
-        <v>627</v>
+        <v>628</v>
       </c>
       <c r="B271" s="1" t="s">
         <v>271</v>
       </c>
       <c r="C271" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
     </row>
     <row r="272" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A272">
-        <v>628</v>
+        <v>629</v>
       </c>
       <c r="B272" s="1" t="s">
         <v>272</v>
       </c>
       <c r="C272" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
     </row>
     <row r="273" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A273">
-        <v>629</v>
+        <v>630</v>
       </c>
       <c r="B273" s="1" t="s">
         <v>273</v>
       </c>
       <c r="C273" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
     </row>
     <row r="274" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A274">
-        <v>630</v>
+        <v>631</v>
       </c>
       <c r="B274" s="1" t="s">
         <v>274</v>
       </c>
       <c r="C274" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
     </row>
     <row r="275" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A275">
-        <v>631</v>
+        <v>632</v>
       </c>
       <c r="B275" s="1" t="s">
         <v>275</v>
       </c>
       <c r="C275" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
     </row>
     <row r="276" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A276">
-        <v>632</v>
+        <v>633</v>
       </c>
       <c r="B276" s="1" t="s">
         <v>276</v>
       </c>
       <c r="C276" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
     </row>
     <row r="277" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A277">
-        <v>633</v>
+        <v>634</v>
       </c>
       <c r="B277" s="1" t="s">
         <v>277</v>
       </c>
       <c r="C277" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
     </row>
     <row r="278" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A278">
-        <v>634</v>
+        <v>635</v>
       </c>
       <c r="B278" s="1" t="s">
         <v>278</v>
       </c>
       <c r="C278" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
     </row>
     <row r="279" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A279">
-        <v>635</v>
+        <v>636</v>
       </c>
       <c r="B279" s="1" t="s">
         <v>279</v>
       </c>
       <c r="C279" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
     </row>
     <row r="280" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A280">
-        <v>636</v>
+        <v>637</v>
       </c>
       <c r="B280" s="1" t="s">
         <v>280</v>
       </c>
       <c r="C280" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
     </row>
     <row r="281" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A281">
-        <v>637</v>
+        <v>638</v>
       </c>
       <c r="B281" s="1" t="s">
         <v>281</v>
       </c>
       <c r="C281" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
     </row>
     <row r="282" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A282">
-        <v>638</v>
+        <v>639</v>
       </c>
       <c r="B282" s="1" t="s">
         <v>282</v>
       </c>
       <c r="C282" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
     </row>
     <row r="283" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A283">
-        <v>639</v>
+        <v>640</v>
       </c>
       <c r="B283" s="1" t="s">
         <v>283</v>
       </c>
       <c r="C283" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
     </row>
     <row r="284" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A284">
-        <v>640</v>
+        <v>641</v>
       </c>
       <c r="B284" s="1" t="s">
         <v>284</v>
       </c>
       <c r="C284" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
     </row>
     <row r="285" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A285">
-        <v>641</v>
+        <v>642</v>
       </c>
       <c r="B285" s="1" t="s">
         <v>285</v>
       </c>
       <c r="C285" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
     </row>
     <row r="286" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A286">
-        <v>642</v>
+        <v>643</v>
       </c>
       <c r="B286" s="1" t="s">
         <v>286</v>
       </c>
       <c r="C286" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
     </row>
     <row r="287" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A287">
-        <v>643</v>
+        <v>644</v>
       </c>
       <c r="B287" s="1" t="s">
         <v>287</v>
       </c>
       <c r="C287" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
     </row>
     <row r="288" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A288">
-        <v>644</v>
+        <v>645</v>
       </c>
       <c r="B288" s="1" t="s">
         <v>288</v>
       </c>
       <c r="C288" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
     </row>
     <row r="289" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A289">
-        <v>645</v>
+        <v>646</v>
       </c>
       <c r="B289" s="1" t="s">
         <v>289</v>
       </c>
       <c r="C289" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
     </row>
     <row r="290" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A290">
-        <v>646</v>
+        <v>647</v>
       </c>
       <c r="B290" s="1" t="s">
         <v>290</v>
       </c>
       <c r="C290" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
     </row>
     <row r="291" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A291">
-        <v>647</v>
+        <v>648</v>
       </c>
       <c r="B291" s="1" t="s">
         <v>291</v>
       </c>
       <c r="C291" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
     </row>
     <row r="292" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A292">
-        <v>648</v>
+        <v>649</v>
       </c>
       <c r="B292" s="1" t="s">
         <v>292</v>
       </c>
       <c r="C292" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
     </row>
     <row r="293" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A293">
-        <v>649</v>
+        <v>650</v>
       </c>
       <c r="B293" s="1" t="s">
         <v>293</v>
       </c>
       <c r="C293" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
     </row>
     <row r="294" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A294">
-        <v>650</v>
+        <v>651</v>
       </c>
       <c r="B294" s="1" t="s">
         <v>294</v>
       </c>
       <c r="C294" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
     </row>
     <row r="295" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A295">
-        <v>651</v>
+        <v>652</v>
       </c>
       <c r="B295" s="1" t="s">
         <v>295</v>
       </c>
       <c r="C295" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
     </row>
     <row r="296" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A296">
-        <v>652</v>
+        <v>653</v>
       </c>
       <c r="B296" s="1" t="s">
         <v>296</v>
       </c>
       <c r="C296" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
     </row>
     <row r="297" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A297">
-        <v>653</v>
+        <v>654</v>
       </c>
       <c r="B297" s="1" t="s">
         <v>297</v>
       </c>
       <c r="C297" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
     </row>
     <row r="298" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A298">
-        <v>654</v>
+        <v>655</v>
       </c>
       <c r="B298" s="1" t="s">
         <v>298</v>
       </c>
       <c r="C298" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
     </row>
     <row r="299" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A299">
-        <v>655</v>
+        <v>656</v>
       </c>
       <c r="B299" s="1" t="s">
         <v>299</v>
       </c>
       <c r="C299" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
     </row>
     <row r="300" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A300">
-        <v>656</v>
+        <v>657</v>
       </c>
       <c r="B300" s="1" t="s">
         <v>300</v>
       </c>
       <c r="C300" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
     </row>
     <row r="301" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A301">
-        <v>657</v>
+        <v>658</v>
       </c>
       <c r="B301" s="1" t="s">
         <v>301</v>
       </c>
       <c r="C301" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
     </row>
     <row r="302" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A302">
-        <v>658</v>
+        <v>659</v>
       </c>
       <c r="B302" s="1" t="s">
         <v>302</v>
       </c>
       <c r="C302" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
     </row>
     <row r="303" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A303">
-        <v>659</v>
+        <v>660</v>
       </c>
       <c r="B303" s="1" t="s">
         <v>303</v>
       </c>
       <c r="C303" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
     </row>
     <row r="304" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A304">
-        <v>660</v>
+        <v>661</v>
       </c>
       <c r="B304" s="1" t="s">
         <v>304</v>
       </c>
       <c r="C304" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
     </row>
     <row r="305" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A305">
-        <v>661</v>
+        <v>662</v>
       </c>
       <c r="B305" s="1" t="s">
         <v>305</v>
       </c>
       <c r="C305" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
     </row>
     <row r="306" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A306">
-        <v>662</v>
+        <v>663</v>
       </c>
       <c r="B306" s="1" t="s">
         <v>306</v>
       </c>
       <c r="C306" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
     </row>
     <row r="307" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A307">
-        <v>663</v>
+        <v>664</v>
       </c>
       <c r="B307" s="1" t="s">
         <v>307</v>
       </c>
       <c r="C307" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
     </row>
     <row r="308" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A308">
-        <v>664</v>
+        <v>665</v>
       </c>
       <c r="B308" s="1" t="s">
         <v>308</v>
       </c>
       <c r="C308" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
     </row>
     <row r="309" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A309">
-        <v>665</v>
+        <v>666</v>
       </c>
       <c r="B309" s="1" t="s">
         <v>309</v>
       </c>
       <c r="C309" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
     </row>
     <row r="310" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A310">
-        <v>666</v>
+        <v>667</v>
       </c>
       <c r="B310" s="1" t="s">
         <v>310</v>
       </c>
       <c r="C310" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
     </row>
     <row r="311" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A311">
-        <v>667</v>
+        <v>668</v>
       </c>
       <c r="B311" s="1" t="s">
         <v>311</v>
       </c>
       <c r="C311" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
     </row>
     <row r="312" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A312">
-        <v>668</v>
+        <v>669</v>
       </c>
       <c r="B312" s="1" t="s">
         <v>312</v>
       </c>
       <c r="C312" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
     </row>
     <row r="313" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A313">
-        <v>669</v>
+        <v>670</v>
       </c>
       <c r="B313" s="1" t="s">
         <v>313</v>
       </c>
       <c r="C313" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
     </row>
     <row r="314" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A314">
-        <v>670</v>
+        <v>671</v>
       </c>
       <c r="B314" s="1" t="s">
         <v>314</v>
       </c>
       <c r="C314" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
     </row>
     <row r="315" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A315">
-        <v>671</v>
+        <v>672</v>
       </c>
       <c r="B315" s="1" t="s">
         <v>315</v>
       </c>
       <c r="C315" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
     </row>
     <row r="316" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A316">
-        <v>672</v>
+        <v>673</v>
       </c>
       <c r="B316" s="1" t="s">
         <v>316</v>
       </c>
       <c r="C316" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
     </row>
     <row r="317" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A317">
-        <v>673</v>
+        <v>674</v>
       </c>
       <c r="B317" s="1" t="s">
         <v>317</v>
       </c>
       <c r="C317" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
     </row>
     <row r="318" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A318">
-        <v>674</v>
+        <v>675</v>
       </c>
       <c r="B318" s="1" t="s">
         <v>318</v>
       </c>
       <c r="C318" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
     </row>
     <row r="319" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A319">
-        <v>675</v>
+        <v>676</v>
       </c>
       <c r="B319" s="1" t="s">
         <v>319</v>
       </c>
       <c r="C319" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
     </row>
     <row r="320" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A320">
-        <v>676</v>
+        <v>677</v>
       </c>
       <c r="B320" s="1" t="s">
         <v>320</v>
       </c>
       <c r="C320" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
     </row>
     <row r="321" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A321">
-        <v>677</v>
+        <v>678</v>
       </c>
       <c r="B321" s="1" t="s">
         <v>321</v>
       </c>
       <c r="C321" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
     </row>
     <row r="322" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A322">
-        <v>678</v>
+        <v>679</v>
       </c>
       <c r="B322" s="1" t="s">
         <v>322</v>
       </c>
       <c r="C322" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
     </row>
     <row r="323" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A323">
-        <v>679</v>
+        <v>680</v>
       </c>
       <c r="B323" s="1" t="s">
         <v>323</v>
       </c>
       <c r="C323" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
     </row>
     <row r="324" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A324">
-        <v>680</v>
+        <v>681</v>
       </c>
       <c r="B324" s="1" t="s">
         <v>324</v>
       </c>
       <c r="C324" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
     </row>
     <row r="325" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A325">
-        <v>681</v>
+        <v>682</v>
       </c>
       <c r="B325" s="1" t="s">
         <v>325</v>
       </c>
       <c r="C325" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
     </row>
     <row r="326" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A326">
-        <v>682</v>
+        <v>683</v>
       </c>
       <c r="B326" s="1" t="s">
         <v>326</v>
       </c>
       <c r="C326" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
     </row>
     <row r="327" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A327">
-        <v>683</v>
+        <v>684</v>
       </c>
       <c r="B327" s="1" t="s">
         <v>327</v>
       </c>
       <c r="C327" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
     </row>
     <row r="328" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A328">
-        <v>684</v>
+        <v>685</v>
       </c>
       <c r="B328" s="1" t="s">
         <v>328</v>
       </c>
       <c r="C328" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
     </row>
     <row r="329" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A329">
-        <v>685</v>
+        <v>686</v>
       </c>
       <c r="B329" s="1" t="s">
         <v>329</v>
       </c>
       <c r="C329" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
     </row>
     <row r="330" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A330">
-        <v>686</v>
+        <v>687</v>
       </c>
       <c r="B330" s="1" t="s">
         <v>330</v>
       </c>
       <c r="C330" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
     </row>
     <row r="331" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A331">
-        <v>687</v>
+        <v>688</v>
       </c>
       <c r="B331" s="1" t="s">
         <v>331</v>
       </c>
       <c r="C331" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
     </row>
     <row r="332" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A332">
-        <v>688</v>
+        <v>689</v>
       </c>
       <c r="B332" s="1" t="s">
         <v>332</v>
       </c>
       <c r="C332" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
     </row>
     <row r="333" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A333">
-        <v>689</v>
+        <v>690</v>
       </c>
       <c r="B333" s="1" t="s">
         <v>333</v>
       </c>
       <c r="C333" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
     </row>
     <row r="334" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A334">
-        <v>690</v>
+        <v>691</v>
       </c>
       <c r="B334" s="1" t="s">
         <v>334</v>
       </c>
       <c r="C334" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
     </row>
     <row r="335" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A335">
-        <v>691</v>
+        <v>692</v>
       </c>
       <c r="B335" s="1" t="s">
         <v>335</v>
       </c>
       <c r="C335" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
     </row>
     <row r="336" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A336">
-        <v>692</v>
+        <v>693</v>
       </c>
       <c r="B336" s="1" t="s">
         <v>336</v>
       </c>
       <c r="C336" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
     </row>
     <row r="337" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A337">
-        <v>693</v>
+        <v>694</v>
       </c>
       <c r="B337" s="1" t="s">
         <v>337</v>
       </c>
       <c r="C337" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
     </row>
     <row r="338" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A338">
-        <v>694</v>
+        <v>695</v>
       </c>
       <c r="B338" s="1" t="s">
         <v>338</v>
       </c>
       <c r="C338" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
     </row>
     <row r="339" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A339">
-        <v>695</v>
+        <v>696</v>
       </c>
       <c r="B339" s="1" t="s">
         <v>339</v>
       </c>
       <c r="C339" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
     </row>
     <row r="340" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A340">
-        <v>696</v>
+        <v>697</v>
       </c>
       <c r="B340" s="1" t="s">
         <v>340</v>
       </c>
       <c r="C340" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
     </row>
     <row r="341" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A341">
-        <v>697</v>
+        <v>698</v>
       </c>
       <c r="B341" s="1" t="s">
         <v>341</v>
       </c>
       <c r="C341" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
     </row>
     <row r="342" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A342">
-        <v>698</v>
+        <v>699</v>
       </c>
       <c r="B342" s="1" t="s">
         <v>342</v>
       </c>
       <c r="C342" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
     </row>
     <row r="343" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A343">
-        <v>699</v>
+        <v>700</v>
       </c>
       <c r="B343" s="1" t="s">
         <v>343</v>
       </c>
       <c r="C343" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
     </row>
     <row r="344" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A344">
-        <v>700</v>
+        <v>701</v>
       </c>
       <c r="B344" s="1" t="s">
         <v>344</v>
       </c>
       <c r="C344" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
     </row>
     <row r="345" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A345">
-        <v>701</v>
+        <v>702</v>
       </c>
       <c r="B345" s="1" t="s">
         <v>345</v>
       </c>
       <c r="C345" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
     </row>
     <row r="346" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A346">
-        <v>702</v>
+        <v>703</v>
       </c>
       <c r="B346" s="1" t="s">
         <v>346</v>
       </c>
       <c r="C346" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
     </row>
     <row r="347" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A347">
-        <v>703</v>
+        <v>704</v>
       </c>
       <c r="B347" s="1" t="s">
         <v>347</v>
       </c>
       <c r="C347" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
     </row>
     <row r="348" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A348">
-        <v>704</v>
+        <v>705</v>
       </c>
       <c r="B348" s="1" t="s">
         <v>348</v>
       </c>
       <c r="C348" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
     </row>
     <row r="349" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A349">
-        <v>705</v>
+        <v>706</v>
       </c>
       <c r="B349" s="1" t="s">
         <v>349</v>
       </c>
       <c r="C349" t="s">
-        <v>359</v>
-      </c>
-    </row>
-    <row r="350" spans="1:3" x14ac:dyDescent="0.25">
+        <v>357</v>
+      </c>
+    </row>
+    <row r="350" spans="1:3" ht="30" x14ac:dyDescent="0.25">
       <c r="A350">
-        <v>706</v>
+        <v>707</v>
       </c>
       <c r="B350" s="1" t="s">
         <v>350</v>
       </c>
       <c r="C350" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
     </row>
     <row r="351" spans="1:3" ht="30" x14ac:dyDescent="0.25">
       <c r="A351">
-        <v>707</v>
+        <v>708</v>
       </c>
       <c r="B351" s="1" t="s">
         <v>351</v>
       </c>
       <c r="C351" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
     </row>
     <row r="352" spans="1:3" ht="30" x14ac:dyDescent="0.25">
       <c r="A352">
-        <v>708</v>
+        <v>709</v>
       </c>
       <c r="B352" s="1" t="s">
         <v>352</v>
       </c>
       <c r="C352" t="s">
-        <v>359</v>
-      </c>
-    </row>
-    <row r="353" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+        <v>357</v>
+      </c>
+    </row>
+    <row r="353" spans="1:3" ht="45" x14ac:dyDescent="0.25">
       <c r="A353">
-        <v>709</v>
+        <v>710</v>
       </c>
       <c r="B353" s="1" t="s">
         <v>353</v>
       </c>
       <c r="C353" t="s">
-        <v>361</v>
+        <v>357</v>
       </c>
     </row>
     <row r="354" spans="1:3" ht="45" x14ac:dyDescent="0.25">
       <c r="A354">
-        <v>710</v>
+        <v>711</v>
       </c>
       <c r="B354" s="1" t="s">
         <v>354</v>
       </c>
       <c r="C354" t="s">
-        <v>361</v>
+        <v>357</v>
       </c>
     </row>
     <row r="355" spans="1:3" ht="45" x14ac:dyDescent="0.25">
       <c r="A355">
-        <v>711</v>
+        <v>712</v>
       </c>
       <c r="B355" s="1" t="s">
         <v>355</v>
       </c>
       <c r="C355" t="s">
-        <v>361</v>
-      </c>
-    </row>
-    <row r="356" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+        <v>357</v>
+      </c>
+    </row>
+    <row r="356" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A356">
-        <v>712</v>
+        <v>713</v>
       </c>
       <c r="B356" s="1" t="s">
         <v>356</v>
       </c>
       <c r="C356" t="s">
-        <v>361</v>
-      </c>
-    </row>
-    <row r="357" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A357">
-        <v>713</v>
-      </c>
-      <c r="B357" s="1" t="s">
-        <v>357</v>
-      </c>
-      <c r="C357" t="s">
-        <v>361</v>
+        <v>357</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>